<commit_message>
corpus: VP66 built — Slide's own face recovered from printed endpoints; Spencer 2.258 vs 2.307/2.30
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/files/rocscience/vp066.xlsx
+++ b/docs/files/rocscience/vp066.xlsx
@@ -15125,7 +15125,7 @@
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
-        <v>-217.0</v>
+        <v>-222.0</v>
       </c>
       <c r="B9" s="3">
         <v>0.0</v>
@@ -15181,7 +15181,7 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>-17.0</v>
+        <v>-15.0</v>
       </c>
       <c r="B10" s="3">
         <v>50.0</v>
@@ -15229,7 +15229,7 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
       <c r="B11" s="3">
         <v>50.0</v>
@@ -15277,7 +15277,7 @@
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
-        <v>217.0</v>
+        <v>222.0</v>
       </c>
       <c r="B12" s="3">
         <v>0.0</v>
@@ -17462,7 +17462,7 @@
         </is>
       </c>
       <c r="E3" s="3">
-        <v>0.0</v>
+        <v>-0.1</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -17920,7 +17920,7 @@
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="3">
-        <v>-217.0</v>
+        <v>-222.0</v>
       </c>
       <c r="C5" s="3">
         <v>0.0</v>
@@ -17946,7 +17946,7 @@
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B6" s="3">
-        <v>-137.0</v>
+        <v>-139.2</v>
       </c>
       <c r="C6" s="3">
         <v>20.0</v>

</xml_diff>